<commit_message>
Auto commit 01-10-2026 22:48:56.94
</commit_message>
<xml_diff>
--- a/Data Base/Global Templates/Filter Point Well.xlsx
+++ b/Data Base/Global Templates/Filter Point Well.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>110mm (4.5") Filterpoint Well Drilling (Code: GWDDR104)</t>
   </si>
@@ -23,6 +23,9 @@
   </si>
   <si>
     <t>Slotting charge for 3m pipe, net, rope, pipe fittings and sundries for Filter Point Well Construction (Code: GWDDR465)</t>
+  </si>
+  <si>
+    <t>PVC end cap 110 mm dia(Code: MR86 - Water Charge and CPOH Added)</t>
   </si>
 </sst>
 </file>
@@ -380,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="60" customWidth="1"/>
@@ -405,9 +408,17 @@
     </row>
     <row r="3" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B4" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>